<commit_message>
add sales Export data
</commit_message>
<xml_diff>
--- a/Sales-Export_2019-2020.xlsx
+++ b/Sales-Export_2019-2020.xlsx
@@ -5,30 +5,31 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\datasets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\datasets\excel dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4960FB6-F0C3-4440-935D-8A62F8FEB34A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08AFCAE-3083-4CA2-BE63-F3C2D47AEB9E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pivot table" sheetId="2" r:id="rId1"/>
     <sheet name="DASHBOARDS" sheetId="3" r:id="rId2"/>
-    <sheet name="Sales-Export_2019-2020" sheetId="1" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
+    <sheet name="Sales-Export_2019-2020" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sales-Export_2019-2020'!$M$1:$R$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sales-Export_2019-2020'!$M$1:$R$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7113" uniqueCount="1182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7119" uniqueCount="1188">
   <si>
     <t>country</t>
   </si>
@@ -3574,6 +3575,24 @@
   </si>
   <si>
     <t>Profit margin %</t>
+  </si>
+  <si>
+    <t>Insights</t>
+  </si>
+  <si>
+    <t>Total sales are 113.36 million, with total cost of 94.36 million and total profit of 18.99 million.</t>
+  </si>
+  <si>
+    <t>There are 1000 total orders, and the average order value is around 113,362.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The overall profit margin is 16.75%, which shows the business is making a moderate profit.</t>
+  </si>
+  <si>
+    <t>From the country-wise analysis, Portugal has the highest sales.</t>
+  </si>
+  <si>
+    <t>Overall, the business is performing well in terms of sales and profit, but there is still scope to improve the profit margin by controlling costs or increasing efficient sales</t>
   </si>
 </sst>
 </file>
@@ -3716,7 +3735,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3905,6 +3924,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4131,7 +4156,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -4155,6 +4180,10 @@
     <xf numFmtId="0" fontId="16" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="34" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -4214,6 +4243,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF48CA36"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -24300,7 +24334,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="HP" refreshedDate="46136.258162731479" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="1000" xr:uid="{00000000-000A-0000-FFFF-FFFF17000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="HP" refreshedDate="46141.573566435189" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="1000" xr:uid="{00000000-000A-0000-FFFF-FFFF17000000}">
   <cacheSource type="worksheet">
     <worksheetSource name="Table3"/>
   </cacheSource>
@@ -37976,7 +38010,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000001000000}" name="PivotTable10" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12" rowHeaderCaption="category">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000001000000}" name="PivotTable10" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12" rowHeaderCaption="category">
   <location ref="G22:H33" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="13">
     <pivotField showAll="0"/>
@@ -38369,7 +38403,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000004000000}" name="PivotTable13" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="17" rowHeaderCaption="manager">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000004000000}" name="PivotTable13" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="17" rowHeaderCaption="manager">
   <location ref="A59:B75" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="13">
     <pivotField showAll="0"/>
@@ -38497,7 +38531,315 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000003000000}" name="PivotTable12" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Year">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="Country">
+  <location ref="A3:B19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="13">
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="16">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="4" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="4" showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="16">
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of  order_value_EUR " fld="1" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000002000000}" name="PivotTable11" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Year">
+  <location ref="A42:B45" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="13">
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="4" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="4" showAll="0"/>
+    <pivotField axis="axisRow" numFmtId="14" showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="5">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="3">
+    <field x="12"/>
+    <field x="11"/>
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of  order_value_EUR " fld="1" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000003000000}" name="PivotTable12" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Year">
   <location ref="H42:I45" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="13">
     <pivotField showAll="0"/>
@@ -38611,8 +38953,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000006000000}" name="PivotTable9" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9" rowHeaderCaption="Country">
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000006000000}" name="PivotTable9" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9" rowHeaderCaption="Country">
   <location ref="A22:B38" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="13">
     <pivotField axis="axisRow" showAll="0" sortType="descending">
@@ -38784,8 +39126,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000005000000}" name="PivotTable8" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Category">
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000005000000}" name="PivotTable8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Category">
   <location ref="G3:H14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="13">
     <pivotField showAll="0"/>
@@ -39177,314 +39519,6 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="Country">
-  <location ref="A3:B19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="13">
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="16">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField dataField="1" numFmtId="4" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="4" showAll="0"/>
-    <pivotField numFmtId="14" showAll="0">
-      <items count="15">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="16">
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of  order_value_EUR " fld="1" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="4" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="5" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000002000000}" name="PivotTable11" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Year">
-  <location ref="A42:B45" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="13">
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="4" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="4" showAll="0"/>
-    <pivotField axis="axisRow" numFmtId="14" showAll="0">
-      <items count="15">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="5">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="3">
-    <field x="12"/>
-    <field x="11"/>
-    <field x="4"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of  order_value_EUR " fld="1" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:K1001" totalsRowShown="0">
   <autoFilter ref="A1:K1001" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
@@ -39810,15 +39844,16 @@
   <dimension ref="A3:I75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.85546875" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -40443,7 +40478,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
     <col min="4" max="4" width="12.42578125" customWidth="1"/>
     <col min="5" max="5" width="16.42578125" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" customWidth="1"/>
@@ -40471,28 +40506,28 @@
     </row>
     <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9">
-        <f>'Sales-Export_2019-2020'!M2</f>
-        <v>0</v>
+        <f>'Sales-Export_2019-2020'!M6</f>
+        <v>113361738.71000001</v>
       </c>
       <c r="B2" s="9">
-        <f>'Sales-Export_2019-2020'!N2</f>
-        <v>0</v>
+        <f>'Sales-Export_2019-2020'!N6</f>
+        <v>94369310.990000054</v>
       </c>
       <c r="C2" s="10">
-        <f>'Sales-Export_2019-2020'!O2</f>
-        <v>0</v>
+        <f>'Sales-Export_2019-2020'!O6</f>
+        <v>18992427.719999999</v>
       </c>
       <c r="D2" s="9">
-        <f>'Sales-Export_2019-2020'!P2</f>
-        <v>0</v>
+        <f>'Sales-Export_2019-2020'!P6</f>
+        <v>1000</v>
       </c>
       <c r="E2" s="9">
-        <f>'Sales-Export_2019-2020'!Q2</f>
-        <v>0</v>
+        <f>'Sales-Export_2019-2020'!Q6</f>
+        <v>113361.73871000001</v>
       </c>
       <c r="F2" s="11">
-        <f>'Sales-Export_2019-2020'!R2</f>
-        <v>0</v>
+        <f>'Sales-Export_2019-2020'!R6</f>
+        <v>0.1675382535247284</v>
       </c>
     </row>
   </sheetData>
@@ -40503,6 +40538,126 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE07306-6FD8-48F4-9682-47C6C9038B89}">
+  <dimension ref="A1:P6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="14" max="14" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>1182</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
+      <c r="N2" s="20"/>
+      <c r="O2" s="20"/>
+      <c r="P2" s="20"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="20"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>1185</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1186</v>
+      </c>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>1187</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="G5:P5"/>
+    <mergeCell ref="A4:P4"/>
+    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A1:P1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -40770,7 +40925,7 @@
         <v>785</v>
       </c>
       <c r="M6" s="17">
-        <f>SUM(Table3 [ order_value_EUR ] )</f>
+        <f>SUM(B:B)</f>
         <v>113361738.71000001</v>
       </c>
       <c r="N6" s="17">

</xml_diff>